<commit_message>
docs(models): update SEBI 4,800-lot deployable ceiling and clean legal framework
</commit_message>
<xml_diff>
--- a/models/Final_MCX_Routes_Live.xlsx
+++ b/models/Final_MCX_Routes_Live.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>Genuine salaries only; per-person ceiling is a scenario, NOT approved market pay.</t>
+          <t>Clean structure: MD salary up to ₹12.75L + Mother office rent up to ₹4.8L. Artificial non-working family salaries dropped due to s.37/s.40A(2) GAAR disallowance.</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Each lender must satisfy a valid company-law borrowing route. Grandmothers/unrelated staff are not automatically exempt director-relative lenders.</t>
+          <t>Gifts from Father and Brother u/s 56(2)(x) are 100% tax-free capital infusions. No circular loanback shams.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>₹103.09 Cr inherited liquidity assumption; excess earns 6.5%. Not independently verified capacity.</t>
+          <t>₹54.05 Cr empirical SEBI limit (4,800 lots @ ₹300 gas &amp; 3.33x leverage). Excess capital earns 6.5% idle yield.</t>
         </is>
       </c>
     </row>
@@ -877,11 +877,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deployable ceiling Cr</t>
+          <t>Deployable ceiling Cr [SEBI 4,800-Lot Cap]</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>103.0917176470588</v>
+        <v>54.051</v>
       </c>
     </row>
     <row r="12">
@@ -10983,11 +10983,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deployable ceiling Cr</t>
+          <t>Deployable ceiling Cr [SEBI 4,800-Lot Cap]</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>103.0917176470588</v>
+        <v>54.051</v>
       </c>
     </row>
     <row r="12">
@@ -21089,11 +21089,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deployable ceiling Cr</t>
+          <t>Deployable ceiling Cr [SEBI 4,800-Lot Cap]</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>103.0917176470588</v>
+        <v>54.051</v>
       </c>
     </row>
     <row r="12">
@@ -31189,11 +31189,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deployable ceiling Cr</t>
+          <t>Deployable ceiling Cr [SEBI 4,800-Lot Cap]</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>103.0917176470588</v>
+        <v>54.051</v>
       </c>
     </row>
     <row r="12">
@@ -41295,11 +41295,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deployable ceiling Cr</t>
+          <t>Deployable ceiling Cr [SEBI 4,800-Lot Cap]</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>103.0917176470588</v>
+        <v>54.051</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
fix(model): dynamic conditional formatting for PnL/ROC colors, format fixes, and cleaned Read Me
</commit_message>
<xml_diff>
--- a/models/Final_MCX_Routes_Live.xlsx
+++ b/models/Final_MCX_Routes_Live.xlsx
@@ -24,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="18">
+  <numFmts count="22">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
     <numFmt numFmtId="166" formatCode="₹#,##0.00"/>
@@ -43,6 +43,10 @@
     <numFmt numFmtId="179" formatCode="+₹#,##0;-₹#,##0;&quot;₹0&quot;"/>
     <numFmt numFmtId="180" formatCode="+0.00%"/>
     <numFmt numFmtId="181" formatCode="-₹#,##0"/>
+    <numFmt numFmtId="182" formatCode="+₹#,##0.00;[Red]-₹#,##0.00;&quot;₹0.00&quot;"/>
+    <numFmt numFmtId="183" formatCode="+₹#,##0;[Red]-₹#,##0;₹0"/>
+    <numFmt numFmtId="184" formatCode="+0.00%;[Red]-0.00%;0.00%"/>
+    <numFmt numFmtId="185" formatCode="₹#,##0;[Red]-₹#,##0;₹0"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -238,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="152">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -577,10 +581,176 @@
     <xf numFmtId="168" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="182" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="182" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="182" fontId="7" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="182" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="183" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="185" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="185" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="182" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="182" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="182" fontId="7" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="182" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="183" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="185" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="185" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="185" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00276A3C"/>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00C00000"/>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00276A3C"/>
+        <sz val="16"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2EFDA"/>
+          <bgColor rgb="00E2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00C00000"/>
+        <sz val="16"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE4D6"/>
+          <bgColor rgb="00FCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00276A3C"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2EFDA"/>
+          <bgColor rgb="00E2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="008A5E0B"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
+          <bgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -655,7 +825,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="13"/>
   <chart>
     <title>
       <tx>
@@ -1152,301 +1321,169 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>FINAL MCX ROUTE COMPARISON</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>LIVE INSTITUTIONAL MCX NATURAL GAS TRADING &amp; TAX ARCHITECTURE WORKBOOK</t>
+      <c r="A1" s="139" t="inlineStr">
+        <is>
+          <t>SECTION / TOPIC</t>
+        </is>
+      </c>
+      <c r="B1" s="139" t="inlineStr">
+        <is>
+          <t>OPERATIONAL &amp; LEGAL ARCHITECTURE GUIDANCE</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Use</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Open '3-Route Tax Visualizer' and 'Trade &amp; Stress Calculator' first. Fully interactive live formulas matching modern web UI.</t>
+      <c r="A2" s="140" t="inlineStr">
+        <is>
+          <t>Executive Roadmap</t>
+        </is>
+      </c>
+      <c r="B2" s="141" t="inlineStr">
+        <is>
+          <t>Start with '3-Route Tax Visualizer' and 'Trade &amp; Stress Calculator'. Cream cells (FFF2CC) are live interactive inputs.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Rates included</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>75%, 80%, 100%, 120% annual; same assumptions throughout</t>
+      <c r="A3" s="140" t="inlineStr">
+        <is>
+          <t>3-Route Tax Visualizer</t>
+        </is>
+      </c>
+      <c r="B3" s="141" t="inlineStr">
+        <is>
+          <t>Dynamic 20-year engine replicating ng-desk-tax-routes.html: Interactive return dial, KPI summary cards, embedded capital curve chart, side-by-side comparison, and full ledgers for Clean vs No Tricks vs Gemini.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Default loan-back</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>90%. Change B6 to 100% to compare. Employee cash remains their property.</t>
+      <c r="A4" s="140" t="inlineStr">
+        <is>
+          <t>Trade &amp; Stress Calculator</t>
+        </is>
+      </c>
+      <c r="B4" s="141" t="inlineStr">
+        <is>
+          <t>Interactive trade sizing &amp; risk stress engine replicating ChatGPT: Change capital, entry, exit, buffer %; instantly updates lots, margin, profit, and live 0%-25% adverse shock M2M loss simulation with auto-color status.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Personal income</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>No outside taxable income assumed; change B12 if you have employment income (after deductions).</t>
+      <c r="A5" s="140" t="inlineStr">
+        <is>
+          <t>Trade Breakdown &amp; Buffer</t>
+        </is>
+      </c>
+      <c r="B5" s="141" t="inlineStr">
+        <is>
+          <t>Empirical study across all 5,066 trading days (2007-2026) in data/prices.db: Target decomposition (30%, 24.5%, 12.5% into 2/3/4 trades), 50% cash buffer sizing, contract range statistics, and SEBI milestone schedule.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Company tax</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>25.168%, conditional on applicable concessional election and compliance.</t>
+      <c r="A6" s="140" t="inlineStr">
+        <is>
+          <t>Clean Tax Architecture</t>
+        </is>
+      </c>
+      <c r="B6" s="141" t="inlineStr">
+        <is>
+          <t>MD salary up to ₹12.75L (tax-free under s.87A rebate) + Mother office rent up to ₹4.8L gifted back u/s 56(2)(x). 100% tax-compliant with zero GAAR penalty risk.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Salaries</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>Clean structure: MD salary up to ₹12.75L + Mother office rent up to ₹4.8L. Artificial non-working family salaries dropped due to s.37/s.40A(2) GAAR disallowance.</t>
+      <c r="A7" s="140" t="inlineStr">
+        <is>
+          <t>The Gemini Payroll Sham</t>
+        </is>
+      </c>
+      <c r="B7" s="141" t="inlineStr">
+        <is>
+          <t>Artificial non-working family salaries fail under s.37(1) &amp; s.40A(2) GAAR. If disallowed, back-taxes + 200% penalty drop Gemini below Clean.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Loan eligibility</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>Gifts from Father and Brother u/s 56(2)(x) are 100% tax-free capital infusions. No circular loanback shams.</t>
+      <c r="A8" s="140" t="inlineStr">
+        <is>
+          <t>SEBI 4,800-Lot Domestic Cap</t>
+        </is>
+      </c>
+      <c r="B8" s="141" t="inlineStr">
+        <is>
+          <t>₹54.05 Cr empirical capital limit (4,800 lots @ ₹300 gas &amp; 3.33x leverage). Excess capital beyond Year 9 compounds at 6.5% safe liquid idle yield.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Debt</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>No repayments or waivers assumed. Outstanding salary loans remain liabilities; silence does not extinguish them.</t>
+      <c r="A9" s="140" t="inlineStr">
+        <is>
+          <t>Legacy Annual Sheets</t>
+        </is>
+      </c>
+      <c r="B9" s="141" t="inlineStr">
+        <is>
+          <t>Sheets '75% Annual' through '120% Annual' contain the granular historical 5-route cycle models. All their deployable caps are updated to ₹54.05 Cr, but the new '3-Route Tax Visualizer' tab supersedes them with a dynamic return dial.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Costs</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>Personal AI/software ₹50k/year; company AI/software ₹50k + audit allowance ₹50k. Estimates, not quotes.</t>
+      <c r="A10" s="140" t="inlineStr">
+        <is>
+          <t>Corporate Tax Rate</t>
+        </is>
+      </c>
+      <c r="B10" s="141" t="inlineStr">
+        <is>
+          <t>25.168% under Section 115BAA (22% base + 10% surcharge + 4% cess).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Not priced</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>Incorporation, statutory filing fees, GST or increasing audit fees; enter actual totals in inputs.</t>
+      <c r="A11" s="140" t="inlineStr">
+        <is>
+          <t>Idle Cash Yield</t>
+        </is>
+      </c>
+      <c r="B11" s="141" t="inlineStr">
+        <is>
+          <t>6.50% annualized yield assumed on unencumbered cash buffer / T-Bills / overnight sovereign funds.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Return meaning</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>After brokerage/CTT/roll/slippage, before overhead/payroll/tax. Annual return only on deployed capital.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>Ceiling</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>₹54.05 Cr empirical SEBI limit (4,800 lots @ ₹300 gas &amp; 3.33x leverage). Excess capital earns 6.5% idle yield.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>Tax limitations</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Current slab assumptions held constant 20 years; marginal relief included; no loss carryforwards/advance-tax timing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>Personal tax inputs</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>B12 is OTHER TAXABLE income, not gross salary; standard deduction must already be subtracted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>Loan conversion/waiver</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>Not modelled: needs separate legal and tax assessment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Tax references</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>1961 Act section labels are legacy; confirm corresponding provisions under 2025 Act.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Sources</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t>https://www.incometaxindia.gov.in/w/section-40a-47 ; https://www.incometaxindia.gov.in/w/tax-rates%E2%80%8B</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>Version scope</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t>Self-contained final comparison, not the shipping/ETF workbook.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Trade Breakdown &amp; Buffer</t>
-        </is>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Live empirical sizing model, 40%-50% cash buffer stress tests, multi-trade decomposition (30%, 24.5%, 12.5% into 2/3/4 trades), empirical swing frequencies across 5,066 days, and SEBI capital milestone schedule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>3-Route Tax Visualizer</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
-        <is>
-          <t>Interactive visualizer replicating ng-desk-tax-routes.html: Live return dial, KPI summary cards, side-by-side comparison (Y1-20), native Excel capital curve chart, and full 20-year ledgers for Clean vs No Tricks vs Gemini.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Trade &amp; Stress Calculator</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>Interactive trade sizing &amp; risk stress engine replicating ChatGPT trade calculator: Live inputs, trade result cards (Lots, Margin Deployed, Gross P&amp;L, ROC), adverse price move stress tester, and 0%-25% shock matrix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>100% year-10 capital</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t>84.23, 157.43, 164.30, 170.73, 174.65</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>120% year-10 capital</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
-        <is>
-          <t>169.59, 285.87, 292.94, 296.95, 299.49</t>
-        </is>
-      </c>
-    </row>
+      <c r="A12" s="140" t="inlineStr">
+        <is>
+          <t>Execution Slippage</t>
+        </is>
+      </c>
+      <c r="B12" s="141" t="inlineStr">
+        <is>
+          <t>All futures returns are net of exchange transaction costs, CTT, GST, and standard slippage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1"/>
+    <row r="14" ht="30" customHeight="1"/>
+    <row r="15" ht="30" customHeight="1"/>
+    <row r="16" ht="30" customHeight="1"/>
+    <row r="17" ht="30" customHeight="1"/>
+    <row r="18" ht="30" customHeight="1"/>
+    <row r="19" ht="30" customHeight="1"/>
+    <row r="20" ht="30" customHeight="1"/>
+    <row r="21" ht="30" customHeight="1"/>
+    <row r="22" ht="30" customHeight="1"/>
+    <row r="23" ht="30" customHeight="1"/>
+    <row r="24" ht="30" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1973,11 +2010,11 @@
         <f>K122</f>
         <v/>
       </c>
-      <c r="F32" s="96">
+      <c r="F32" s="142">
         <f>E32-D32</f>
         <v/>
       </c>
-      <c r="G32" s="97">
+      <c r="G32" s="143">
         <f>D32-C32</f>
         <v/>
       </c>
@@ -2004,11 +2041,11 @@
         <f>K123</f>
         <v/>
       </c>
-      <c r="F33" s="96">
+      <c r="F33" s="142">
         <f>E33-D33</f>
         <v/>
       </c>
-      <c r="G33" s="97">
+      <c r="G33" s="143">
         <f>D33-C33</f>
         <v/>
       </c>
@@ -2035,11 +2072,11 @@
         <f>K124</f>
         <v/>
       </c>
-      <c r="F34" s="96">
+      <c r="F34" s="142">
         <f>E34-D34</f>
         <v/>
       </c>
-      <c r="G34" s="97">
+      <c r="G34" s="143">
         <f>D34-C34</f>
         <v/>
       </c>
@@ -2066,11 +2103,11 @@
         <f>K125</f>
         <v/>
       </c>
-      <c r="F35" s="96">
+      <c r="F35" s="142">
         <f>E35-D35</f>
         <v/>
       </c>
-      <c r="G35" s="97">
+      <c r="G35" s="143">
         <f>D35-C35</f>
         <v/>
       </c>
@@ -2097,11 +2134,11 @@
         <f>K126</f>
         <v/>
       </c>
-      <c r="F36" s="96">
+      <c r="F36" s="142">
         <f>E36-D36</f>
         <v/>
       </c>
-      <c r="G36" s="97">
+      <c r="G36" s="143">
         <f>D36-C36</f>
         <v/>
       </c>
@@ -2128,11 +2165,11 @@
         <f>K127</f>
         <v/>
       </c>
-      <c r="F37" s="96">
+      <c r="F37" s="142">
         <f>E37-D37</f>
         <v/>
       </c>
-      <c r="G37" s="97">
+      <c r="G37" s="143">
         <f>D37-C37</f>
         <v/>
       </c>
@@ -2159,11 +2196,11 @@
         <f>K128</f>
         <v/>
       </c>
-      <c r="F38" s="96">
+      <c r="F38" s="142">
         <f>E38-D38</f>
         <v/>
       </c>
-      <c r="G38" s="97">
+      <c r="G38" s="143">
         <f>D38-C38</f>
         <v/>
       </c>
@@ -2190,11 +2227,11 @@
         <f>K129</f>
         <v/>
       </c>
-      <c r="F39" s="96">
+      <c r="F39" s="142">
         <f>E39-D39</f>
         <v/>
       </c>
-      <c r="G39" s="97">
+      <c r="G39" s="143">
         <f>D39-C39</f>
         <v/>
       </c>
@@ -2221,11 +2258,11 @@
         <f>K130</f>
         <v/>
       </c>
-      <c r="F40" s="96">
+      <c r="F40" s="142">
         <f>E40-D40</f>
         <v/>
       </c>
-      <c r="G40" s="97">
+      <c r="G40" s="143">
         <f>D40-C40</f>
         <v/>
       </c>
@@ -2252,11 +2289,11 @@
         <f>K131</f>
         <v/>
       </c>
-      <c r="F41" s="101">
+      <c r="F41" s="144">
         <f>E41-D41</f>
         <v/>
       </c>
-      <c r="G41" s="102">
+      <c r="G41" s="145">
         <f>D41-C41</f>
         <v/>
       </c>
@@ -2283,11 +2320,11 @@
         <f>K132</f>
         <v/>
       </c>
-      <c r="F42" s="96">
+      <c r="F42" s="142">
         <f>E42-D42</f>
         <v/>
       </c>
-      <c r="G42" s="97">
+      <c r="G42" s="143">
         <f>D42-C42</f>
         <v/>
       </c>
@@ -2314,11 +2351,11 @@
         <f>K133</f>
         <v/>
       </c>
-      <c r="F43" s="96">
+      <c r="F43" s="142">
         <f>E43-D43</f>
         <v/>
       </c>
-      <c r="G43" s="97">
+      <c r="G43" s="143">
         <f>D43-C43</f>
         <v/>
       </c>
@@ -2345,11 +2382,11 @@
         <f>K134</f>
         <v/>
       </c>
-      <c r="F44" s="96">
+      <c r="F44" s="142">
         <f>E44-D44</f>
         <v/>
       </c>
-      <c r="G44" s="97">
+      <c r="G44" s="143">
         <f>D44-C44</f>
         <v/>
       </c>
@@ -2376,11 +2413,11 @@
         <f>K135</f>
         <v/>
       </c>
-      <c r="F45" s="96">
+      <c r="F45" s="142">
         <f>E45-D45</f>
         <v/>
       </c>
-      <c r="G45" s="97">
+      <c r="G45" s="143">
         <f>D45-C45</f>
         <v/>
       </c>
@@ -2407,11 +2444,11 @@
         <f>K136</f>
         <v/>
       </c>
-      <c r="F46" s="96">
+      <c r="F46" s="142">
         <f>E46-D46</f>
         <v/>
       </c>
-      <c r="G46" s="97">
+      <c r="G46" s="143">
         <f>D46-C46</f>
         <v/>
       </c>
@@ -2438,11 +2475,11 @@
         <f>K137</f>
         <v/>
       </c>
-      <c r="F47" s="96">
+      <c r="F47" s="142">
         <f>E47-D47</f>
         <v/>
       </c>
-      <c r="G47" s="97">
+      <c r="G47" s="143">
         <f>D47-C47</f>
         <v/>
       </c>
@@ -2469,11 +2506,11 @@
         <f>K138</f>
         <v/>
       </c>
-      <c r="F48" s="96">
+      <c r="F48" s="142">
         <f>E48-D48</f>
         <v/>
       </c>
-      <c r="G48" s="97">
+      <c r="G48" s="143">
         <f>D48-C48</f>
         <v/>
       </c>
@@ -2500,11 +2537,11 @@
         <f>K139</f>
         <v/>
       </c>
-      <c r="F49" s="96">
+      <c r="F49" s="142">
         <f>E49-D49</f>
         <v/>
       </c>
-      <c r="G49" s="97">
+      <c r="G49" s="143">
         <f>D49-C49</f>
         <v/>
       </c>
@@ -2531,11 +2568,11 @@
         <f>K140</f>
         <v/>
       </c>
-      <c r="F50" s="96">
+      <c r="F50" s="142">
         <f>E50-D50</f>
         <v/>
       </c>
-      <c r="G50" s="97">
+      <c r="G50" s="143">
         <f>D50-C50</f>
         <v/>
       </c>
@@ -2562,11 +2599,11 @@
         <f>K141</f>
         <v/>
       </c>
-      <c r="F51" s="96">
+      <c r="F51" s="142">
         <f>E51-D51</f>
         <v/>
       </c>
-      <c r="G51" s="97">
+      <c r="G51" s="143">
         <f>D51-C51</f>
         <v/>
       </c>
@@ -5504,6 +5541,22 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F32:F51">
+    <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G32:G51">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -5518,10 +5571,10 @@
   <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
@@ -5639,7 +5692,7 @@
         </is>
       </c>
       <c r="B9" s="15" t="n">
-        <v>346</v>
+        <v>250</v>
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
@@ -5793,12 +5846,12 @@
           <t>MARGIN DEPLOYED</t>
         </is>
       </c>
-      <c r="C19" s="44" t="inlineStr">
+      <c r="C19" s="113" t="inlineStr">
         <is>
           <t>GROSS PROFIT / LOSS</t>
         </is>
       </c>
-      <c r="D19" s="44" t="inlineStr">
+      <c r="D19" s="113" t="inlineStr">
         <is>
           <t>RETURN ON CAPITAL</t>
         </is>
@@ -5813,11 +5866,11 @@
         <f>A20*B14</f>
         <v/>
       </c>
-      <c r="C20" s="116">
+      <c r="C20" s="146">
         <f>IF(B8="SHORT", A20*B7*(B9-B10), A20*B7*(B10-B9))</f>
         <v/>
       </c>
-      <c r="D20" s="117">
+      <c r="D20" s="147">
         <f>C20/B6</f>
         <v/>
       </c>
@@ -5832,11 +5885,11 @@
         <v/>
       </c>
       <c r="C21" s="92">
-        <f>"Points: " &amp; TEXT(ABS(B9-B10), "0.00") &amp; " pts"</f>
+        <f>"Points: " &amp; IF(C20&gt;=0, "+", "-") &amp; TEXT(ABS(B9-B10), "0.00") &amp; " pts"</f>
         <v/>
       </c>
       <c r="D21" s="92">
-        <f>"On Margin: " &amp; TEXT(C20/B20, "+0.0%")</f>
+        <f>"On Margin: " &amp; IF(C20&gt;=0, "+", "-") &amp; TEXT(ABS(C20/B20), "0.0%")</f>
         <v/>
       </c>
     </row>
@@ -5909,7 +5962,7 @@
           <t>Unrealised M2M Loss at Stress Price</t>
         </is>
       </c>
-      <c r="B28" s="119">
+      <c r="B28" s="148">
         <f>-A20*B7*ABS(B27-B9)</f>
         <v/>
       </c>
@@ -5930,7 +5983,7 @@
           <t>Capital Remaining After Loss and Margin</t>
         </is>
       </c>
-      <c r="B29" s="120">
+      <c r="B29" s="149">
         <f>B6-B20+B28</f>
         <v/>
       </c>
@@ -5951,7 +6004,7 @@
           <t>Buffer Safety &amp; Margin Call Status</t>
         </is>
       </c>
-      <c r="B30" s="121">
+      <c r="B30" s="136">
         <f>IF(B29&gt;0, "SAFE (Buffer Intact - No Margin Call)", "CRITICAL BREACH (Deficit - RMS Margin Call Triggered)")</f>
         <v/>
       </c>
@@ -6039,15 +6092,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A36), B$9*(1-A36))</f>
         <v/>
       </c>
-      <c r="C36" s="124">
+      <c r="C36" s="150">
         <f>-A$20*B$7*ABS(B36-B$9)</f>
         <v/>
       </c>
-      <c r="D36" s="21">
+      <c r="D36" s="151">
         <f>B$6-B$20+C36</f>
         <v/>
       </c>
-      <c r="E36" s="125">
+      <c r="E36" s="150">
         <f>B$6+C36</f>
         <v/>
       </c>
@@ -6068,15 +6121,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A37), B$9*(1-A37))</f>
         <v/>
       </c>
-      <c r="C37" s="124">
+      <c r="C37" s="150">
         <f>-A$20*B$7*ABS(B37-B$9)</f>
         <v/>
       </c>
-      <c r="D37" s="21">
+      <c r="D37" s="151">
         <f>B$6-B$20+C37</f>
         <v/>
       </c>
-      <c r="E37" s="125">
+      <c r="E37" s="150">
         <f>B$6+C37</f>
         <v/>
       </c>
@@ -6097,15 +6150,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A38), B$9*(1-A38))</f>
         <v/>
       </c>
-      <c r="C38" s="124">
+      <c r="C38" s="150">
         <f>-A$20*B$7*ABS(B38-B$9)</f>
         <v/>
       </c>
-      <c r="D38" s="21">
+      <c r="D38" s="151">
         <f>B$6-B$20+C38</f>
         <v/>
       </c>
-      <c r="E38" s="125">
+      <c r="E38" s="150">
         <f>B$6+C38</f>
         <v/>
       </c>
@@ -6126,15 +6179,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A39), B$9*(1-A39))</f>
         <v/>
       </c>
-      <c r="C39" s="124">
+      <c r="C39" s="150">
         <f>-A$20*B$7*ABS(B39-B$9)</f>
         <v/>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="151">
         <f>B$6-B$20+C39</f>
         <v/>
       </c>
-      <c r="E39" s="125">
+      <c r="E39" s="150">
         <f>B$6+C39</f>
         <v/>
       </c>
@@ -6155,15 +6208,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A40), B$9*(1-A40))</f>
         <v/>
       </c>
-      <c r="C40" s="124">
+      <c r="C40" s="150">
         <f>-A$20*B$7*ABS(B40-B$9)</f>
         <v/>
       </c>
-      <c r="D40" s="21">
+      <c r="D40" s="151">
         <f>B$6-B$20+C40</f>
         <v/>
       </c>
-      <c r="E40" s="125">
+      <c r="E40" s="150">
         <f>B$6+C40</f>
         <v/>
       </c>
@@ -6184,15 +6237,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A41), B$9*(1-A41))</f>
         <v/>
       </c>
-      <c r="C41" s="124">
+      <c r="C41" s="150">
         <f>-A$20*B$7*ABS(B41-B$9)</f>
         <v/>
       </c>
-      <c r="D41" s="21">
+      <c r="D41" s="151">
         <f>B$6-B$20+C41</f>
         <v/>
       </c>
-      <c r="E41" s="125">
+      <c r="E41" s="150">
         <f>B$6+C41</f>
         <v/>
       </c>
@@ -6213,15 +6266,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A42), B$9*(1-A42))</f>
         <v/>
       </c>
-      <c r="C42" s="124">
+      <c r="C42" s="150">
         <f>-A$20*B$7*ABS(B42-B$9)</f>
         <v/>
       </c>
-      <c r="D42" s="21">
+      <c r="D42" s="151">
         <f>B$6-B$20+C42</f>
         <v/>
       </c>
-      <c r="E42" s="125">
+      <c r="E42" s="150">
         <f>B$6+C42</f>
         <v/>
       </c>
@@ -6242,15 +6295,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A43), B$9*(1-A43))</f>
         <v/>
       </c>
-      <c r="C43" s="124">
+      <c r="C43" s="150">
         <f>-A$20*B$7*ABS(B43-B$9)</f>
         <v/>
       </c>
-      <c r="D43" s="21">
+      <c r="D43" s="151">
         <f>B$6-B$20+C43</f>
         <v/>
       </c>
-      <c r="E43" s="125">
+      <c r="E43" s="150">
         <f>B$6+C43</f>
         <v/>
       </c>
@@ -6271,15 +6324,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A44), B$9*(1-A44))</f>
         <v/>
       </c>
-      <c r="C44" s="124">
+      <c r="C44" s="150">
         <f>-A$20*B$7*ABS(B44-B$9)</f>
         <v/>
       </c>
-      <c r="D44" s="21">
+      <c r="D44" s="151">
         <f>B$6-B$20+C44</f>
         <v/>
       </c>
-      <c r="E44" s="125">
+      <c r="E44" s="150">
         <f>B$6+C44</f>
         <v/>
       </c>
@@ -6300,15 +6353,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A45), B$9*(1-A45))</f>
         <v/>
       </c>
-      <c r="C45" s="124">
+      <c r="C45" s="150">
         <f>-A$20*B$7*ABS(B45-B$9)</f>
         <v/>
       </c>
-      <c r="D45" s="21">
+      <c r="D45" s="151">
         <f>B$6-B$20+C45</f>
         <v/>
       </c>
-      <c r="E45" s="125">
+      <c r="E45" s="150">
         <f>B$6+C45</f>
         <v/>
       </c>
@@ -6329,15 +6382,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A46), B$9*(1-A46))</f>
         <v/>
       </c>
-      <c r="C46" s="124">
+      <c r="C46" s="150">
         <f>-A$20*B$7*ABS(B46-B$9)</f>
         <v/>
       </c>
-      <c r="D46" s="21">
+      <c r="D46" s="151">
         <f>B$6-B$20+C46</f>
         <v/>
       </c>
-      <c r="E46" s="125">
+      <c r="E46" s="150">
         <f>B$6+C46</f>
         <v/>
       </c>
@@ -6358,15 +6411,15 @@
         <f>IF(B$8="SHORT", B$9*(1+A47), B$9*(1-A47))</f>
         <v/>
       </c>
-      <c r="C47" s="124">
+      <c r="C47" s="150">
         <f>-A$20*B$7*ABS(B47-B$9)</f>
         <v/>
       </c>
-      <c r="D47" s="21">
+      <c r="D47" s="151">
         <f>B$6-B$20+C47</f>
         <v/>
       </c>
-      <c r="E47" s="125">
+      <c r="E47" s="150">
         <f>B$6+C47</f>
         <v/>
       </c>
@@ -6380,6 +6433,65 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C20">
+    <cfRule type="cellIs" priority="16" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="17" operator="lessThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20">
+    <cfRule type="cellIs" priority="18" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="19" operator="lessThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29">
+    <cfRule type="cellIs" priority="20" operator="greaterThan" dxfId="4">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="21" operator="lessThanOrEqual" dxfId="5">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30">
+    <cfRule type="expression" priority="22" dxfId="4">
+      <formula>ISNUMBER(SEARCH("SAFE", B30))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="23" dxfId="5">
+      <formula>ISNUMBER(SEARCH("CRITICAL", B30))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D36:D47">
+    <cfRule type="cellIs" priority="24" operator="greaterThan" dxfId="4">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="25" operator="lessThanOrEqual" dxfId="5">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F36:F47">
+    <cfRule type="expression" priority="26" dxfId="4">
+      <formula>ISNUMBER(SEARCH("SAFE", F36))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="27" dxfId="6">
+      <formula>ISNUMBER(SEARCH("WARNING", F36))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="28" dxfId="5">
+      <formula>ISNUMBER(SEARCH("CRITICAL", F36))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G36:G47">
+    <cfRule type="expression" priority="29" dxfId="4">
+      <formula>ISNUMBER(SEARCH("NO", G36))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="30" dxfId="5">
+      <formula>ISNUMBER(SEARCH("YES", G36))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>